<commit_message>
Update the marks of the owner for the test of decision 0042
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TnghEw2ou31QVRW6aTsXeq
</commit_message>
<xml_diff>
--- a/marking/test-0024-round1.xlsx
+++ b/marking/test-0024-round1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\triggger\ccar-f-mock-generator\marking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3123F1EA-26EE-44EB-9721-7803C1BB60AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7330D0AF-67D5-43FF-9AC3-D679AA6D5C18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31830" yWindow="3030" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Marks" sheetId="1" r:id="rId1"/>
@@ -405,7 +405,7 @@
     <t>bad</t>
   </si>
   <si>
-    <t>The question is confusing and needs calrification.</t>
+    <t>The question is confusing and needs calrification. I had to read the question more than one time. Use one name for the actor, not 'the subagent' and 'Claude'. Make the sentences shorter. Do not change what the question tests, and do not say directly that the search result is missing.</t>
   </si>
 </sst>
 </file>

</xml_diff>